<commit_message>
feat: Establish initial dashboard framework by adding input section layout, configuration constants, diagnostic data files, and a visualization script.
</commit_message>
<xml_diff>
--- a/data/DRM System Diagnostic Assessment - Template.xlsx
+++ b/data/DRM System Diagnostic Assessment - Template.xlsx
@@ -744,16 +744,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -761,19 +765,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -781,23 +785,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -841,11 +845,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,23 +869,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -893,19 +897,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -921,7 +925,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -933,15 +937,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -953,11 +957,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1219,1132 +1223,1132 @@
   <dimension ref="B2:AY198"/>
   <sheetFormatPr defaultColWidth="8.6015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="87.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="19.61"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="6" style="2" width="6.78"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="2" width="11.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="87.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="19.61"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="6" style="3" width="6.78"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="3" width="11.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20.55"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6"/>
-      <c r="G7" s="2" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="7"/>
+      <c r="G7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="7" t="n">
+      <c r="B8" s="9"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="8" t="n">
         <f aca="false">COUNTBLANK(E15:E61)</f>
         <v>47</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
-      <c r="U8" s="12"/>
-      <c r="V8" s="12"/>
-      <c r="W8" s="12"/>
-      <c r="X8" s="12"/>
-      <c r="Y8" s="12"/>
-      <c r="Z8" s="12"/>
-      <c r="AA8" s="12"/>
-      <c r="AB8" s="12"/>
-      <c r="AC8" s="12"/>
-      <c r="AD8" s="12"/>
-      <c r="AE8" s="12"/>
-      <c r="AF8" s="12"/>
-      <c r="AG8" s="12"/>
-      <c r="AH8" s="12"/>
-      <c r="AI8" s="12"/>
-      <c r="AJ8" s="12"/>
-      <c r="AK8" s="12"/>
-      <c r="AL8" s="12"/>
-      <c r="AM8" s="12"/>
-      <c r="AN8" s="12"/>
-      <c r="AO8" s="12"/>
-      <c r="AP8" s="12"/>
-      <c r="AQ8" s="12"/>
-      <c r="AR8" s="12"/>
-      <c r="AS8" s="12"/>
-      <c r="AT8" s="12"/>
-      <c r="AU8" s="12"/>
-      <c r="AV8" s="12"/>
-      <c r="AW8" s="12"/>
-      <c r="AX8" s="12"/>
-      <c r="AY8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="13"/>
+      <c r="S8" s="13"/>
+      <c r="T8" s="13"/>
+      <c r="U8" s="13"/>
+      <c r="V8" s="13"/>
+      <c r="W8" s="13"/>
+      <c r="X8" s="13"/>
+      <c r="Y8" s="13"/>
+      <c r="Z8" s="13"/>
+      <c r="AA8" s="13"/>
+      <c r="AB8" s="13"/>
+      <c r="AC8" s="13"/>
+      <c r="AD8" s="13"/>
+      <c r="AE8" s="13"/>
+      <c r="AF8" s="13"/>
+      <c r="AG8" s="13"/>
+      <c r="AH8" s="13"/>
+      <c r="AI8" s="13"/>
+      <c r="AJ8" s="13"/>
+      <c r="AK8" s="13"/>
+      <c r="AL8" s="13"/>
+      <c r="AM8" s="13"/>
+      <c r="AN8" s="13"/>
+      <c r="AO8" s="13"/>
+      <c r="AP8" s="13"/>
+      <c r="AQ8" s="13"/>
+      <c r="AR8" s="13"/>
+      <c r="AS8" s="13"/>
+      <c r="AT8" s="13"/>
+      <c r="AU8" s="13"/>
+      <c r="AV8" s="13"/>
+      <c r="AW8" s="13"/>
+      <c r="AX8" s="13"/>
+      <c r="AY8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="12"/>
-      <c r="W9" s="12"/>
-      <c r="X9" s="12"/>
-      <c r="Y9" s="12"/>
-      <c r="Z9" s="12"/>
-      <c r="AA9" s="12"/>
-      <c r="AB9" s="12"/>
-      <c r="AC9" s="12"/>
-      <c r="AD9" s="12"/>
-      <c r="AE9" s="12"/>
-      <c r="AF9" s="12"/>
-      <c r="AG9" s="12"/>
-      <c r="AH9" s="12"/>
-      <c r="AI9" s="12"/>
-      <c r="AJ9" s="12"/>
-      <c r="AK9" s="12"/>
-      <c r="AL9" s="12"/>
-      <c r="AM9" s="12"/>
-      <c r="AN9" s="12"/>
-      <c r="AO9" s="12"/>
-      <c r="AP9" s="12"/>
-      <c r="AQ9" s="12"/>
-      <c r="AR9" s="12"/>
-      <c r="AS9" s="12"/>
-      <c r="AT9" s="12"/>
-      <c r="AU9" s="12"/>
-      <c r="AV9" s="12"/>
-      <c r="AW9" s="12"/>
-      <c r="AX9" s="12"/>
-      <c r="AY9" s="12"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="13"/>
+      <c r="S9" s="13"/>
+      <c r="T9" s="13"/>
+      <c r="U9" s="13"/>
+      <c r="V9" s="13"/>
+      <c r="W9" s="13"/>
+      <c r="X9" s="13"/>
+      <c r="Y9" s="13"/>
+      <c r="Z9" s="13"/>
+      <c r="AA9" s="13"/>
+      <c r="AB9" s="13"/>
+      <c r="AC9" s="13"/>
+      <c r="AD9" s="13"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="13"/>
+      <c r="AG9" s="13"/>
+      <c r="AH9" s="13"/>
+      <c r="AI9" s="13"/>
+      <c r="AJ9" s="13"/>
+      <c r="AK9" s="13"/>
+      <c r="AL9" s="13"/>
+      <c r="AM9" s="13"/>
+      <c r="AN9" s="13"/>
+      <c r="AO9" s="13"/>
+      <c r="AP9" s="13"/>
+      <c r="AQ9" s="13"/>
+      <c r="AR9" s="13"/>
+      <c r="AS9" s="13"/>
+      <c r="AT9" s="13"/>
+      <c r="AU9" s="13"/>
+      <c r="AV9" s="13"/>
+      <c r="AW9" s="13"/>
+      <c r="AX9" s="13"/>
+      <c r="AY9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="14" t="str">
+      <c r="B10" s="15" t="str">
         <f aca="false">IF(G8&gt;0,_xlfn.CONCAT("Please complete asessment to proceed. Remaining questions: ",G8), _xlfn.TEXTJOIN(";",FALSE(),H15:H61))</f>
         <v>Please complete asessment to proceed. Remaining questions: 47</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="11" t="s">
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="12"/>
-      <c r="W10" s="12"/>
-      <c r="X10" s="12"/>
-      <c r="Y10" s="12"/>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="12"/>
-      <c r="AB10" s="12"/>
-      <c r="AC10" s="12"/>
-      <c r="AD10" s="12"/>
-      <c r="AE10" s="12"/>
-      <c r="AF10" s="12"/>
-      <c r="AG10" s="12"/>
-      <c r="AH10" s="12"/>
-      <c r="AI10" s="12"/>
-      <c r="AJ10" s="12"/>
-      <c r="AK10" s="12"/>
-      <c r="AL10" s="12"/>
-      <c r="AM10" s="12"/>
-      <c r="AN10" s="12"/>
-      <c r="AO10" s="12"/>
-      <c r="AP10" s="12"/>
-      <c r="AQ10" s="12"/>
-      <c r="AR10" s="12"/>
-      <c r="AS10" s="12"/>
-      <c r="AT10" s="12"/>
-      <c r="AU10" s="12"/>
-      <c r="AV10" s="12"/>
-      <c r="AW10" s="12"/>
-      <c r="AX10" s="12"/>
-      <c r="AY10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="13"/>
+      <c r="AI10" s="13"/>
+      <c r="AJ10" s="13"/>
+      <c r="AK10" s="13"/>
+      <c r="AL10" s="13"/>
+      <c r="AM10" s="13"/>
+      <c r="AN10" s="13"/>
+      <c r="AO10" s="13"/>
+      <c r="AP10" s="13"/>
+      <c r="AQ10" s="13"/>
+      <c r="AR10" s="13"/>
+      <c r="AS10" s="13"/>
+      <c r="AT10" s="13"/>
+      <c r="AU10" s="13"/>
+      <c r="AV10" s="13"/>
+      <c r="AW10" s="13"/>
+      <c r="AX10" s="13"/>
+      <c r="AY10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="7"/>
+      <c r="B11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="18" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="7"/>
+      <c r="B13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="24" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="29" t="s">
+      <c r="E15" s="28"/>
+      <c r="F15" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="2" t="str">
+      <c r="H15" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G15,E15,F15)</f>
         <v>Q1,,1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="24"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25" t="s">
+      <c r="B16" s="25"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="30"/>
-      <c r="F16" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="E16" s="31"/>
+      <c r="F16" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H16" s="2" t="str">
+      <c r="H16" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G16,E16,F16)</f>
         <v>Q2,,1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="24"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="26" t="s">
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="27"/>
-      <c r="F17" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G17" s="29" t="s">
+      <c r="E17" s="28"/>
+      <c r="F17" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="2" t="str">
+      <c r="H17" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G17,E17,F17)</f>
-        <v>Q3,,0.5</v>
+        <v>Q3,,1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="24"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25" t="s">
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="30"/>
-      <c r="F18" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G18" s="2" t="s">
+      <c r="E18" s="31"/>
+      <c r="F18" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="H18" s="2" t="str">
+      <c r="H18" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G18,E18,F18)</f>
-        <v>Q4,,0.5</v>
+        <v>Q4,,1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="24"/>
-      <c r="C19" s="32" t="s">
+      <c r="B19" s="25"/>
+      <c r="C19" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="29" t="s">
+      <c r="E19" s="28"/>
+      <c r="F19" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="2" t="str">
+      <c r="H19" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G19,E19,F19)</f>
         <v>Q5,,1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="24"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32" t="s">
+      <c r="B20" s="25"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="30"/>
-      <c r="F20" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="2" t="s">
+      <c r="E20" s="31"/>
+      <c r="F20" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="2" t="str">
+      <c r="H20" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G20,E20,F20)</f>
         <v>Q6,,1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C21" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="35" t="s">
+      <c r="D21" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="E21" s="27"/>
-      <c r="F21" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="29" t="s">
+      <c r="E21" s="28"/>
+      <c r="F21" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="H21" s="2" t="str">
+      <c r="H21" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G21,E21,F21)</f>
         <v>Q7,,1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="25" t="s">
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="30"/>
-      <c r="F22" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G22" s="2" t="s">
+      <c r="E22" s="31"/>
+      <c r="F22" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H22" s="2" t="str">
+      <c r="H22" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G22,E22,F22)</f>
-        <v>Q8,,0.5</v>
+        <v>Q8,,1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="26" t="s">
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G23" s="29" t="s">
+      <c r="E23" s="28"/>
+      <c r="F23" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="H23" s="2" t="str">
+      <c r="H23" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G23,E23,F23)</f>
-        <v>Q9,,0.5</v>
+        <v>Q9,,1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="37" t="s">
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="30"/>
-      <c r="F24" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="2" t="s">
+      <c r="E24" s="31"/>
+      <c r="F24" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H24" s="2" t="str">
+      <c r="H24" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G24,E24,F24)</f>
         <v>Q10,,1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="40" t="s">
+      <c r="C25" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="29" t="s">
+      <c r="E25" s="28"/>
+      <c r="F25" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="H25" s="2" t="str">
+      <c r="H25" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G25,E25,F25)</f>
         <v>Q11,,1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="39"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="25" t="s">
+      <c r="B26" s="40"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="E26" s="30"/>
-      <c r="F26" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G26" s="2" t="s">
+      <c r="E26" s="31"/>
+      <c r="F26" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="2" t="str">
+      <c r="H26" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G26,E26,F26)</f>
-        <v>Q12,,0.5</v>
+        <v>Q12,,1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="39"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="26" t="s">
+      <c r="B27" s="40"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="27"/>
-      <c r="F27" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G27" s="29" t="s">
+      <c r="E27" s="28"/>
+      <c r="F27" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="H27" s="2" t="str">
+      <c r="H27" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G27,E27,F27)</f>
-        <v>Q13,,0.5</v>
+        <v>Q13,,1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="39"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="25" t="s">
+      <c r="B28" s="40"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="E28" s="30"/>
-      <c r="F28" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="2" t="s">
+      <c r="E28" s="31"/>
+      <c r="F28" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="H28" s="2" t="str">
+      <c r="H28" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G28,E28,F28)</f>
         <v>Q14,,1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="39"/>
-      <c r="C29" s="25" t="s">
+      <c r="B29" s="40"/>
+      <c r="C29" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="D29" s="26" t="s">
+      <c r="D29" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E29" s="27"/>
-      <c r="F29" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="29" t="s">
+      <c r="E29" s="28"/>
+      <c r="F29" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="H29" s="2" t="str">
+      <c r="H29" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G29,E29,F29)</f>
         <v>Q15,,1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="39"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25" t="s">
+      <c r="B30" s="40"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="30"/>
-      <c r="F30" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="2" t="s">
+      <c r="E30" s="31"/>
+      <c r="F30" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="H30" s="2" t="str">
+      <c r="H30" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G30,E30,F30)</f>
         <v>Q16,,1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="39"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="26" t="s">
+      <c r="B31" s="40"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="E31" s="27"/>
-      <c r="F31" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="29" t="s">
+      <c r="E31" s="28"/>
+      <c r="F31" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="H31" s="2" t="str">
+      <c r="H31" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G31,E31,F31)</f>
         <v>Q17,,1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="39"/>
-      <c r="C32" s="32" t="s">
+      <c r="B32" s="40"/>
+      <c r="C32" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="E32" s="30"/>
-      <c r="F32" s="31" t="n">
+      <c r="E32" s="31"/>
+      <c r="F32" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="H32" s="2" t="str">
+      <c r="H32" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G32,E32,F32)</f>
         <v>Q18,,0.25</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="39"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="43" t="s">
+      <c r="B33" s="40"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="E33" s="27"/>
-      <c r="F33" s="28" t="n">
+      <c r="E33" s="28"/>
+      <c r="F33" s="29" t="n">
         <v>0.25</v>
       </c>
-      <c r="G33" s="29" t="s">
+      <c r="G33" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="H33" s="2" t="str">
+      <c r="H33" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G33,E33,F33)</f>
         <v>Q19,,0.25</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="39"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="44" t="s">
+      <c r="B34" s="40"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="E34" s="30"/>
-      <c r="F34" s="31" t="n">
+      <c r="E34" s="31"/>
+      <c r="F34" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H34" s="2" t="str">
+      <c r="H34" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G34,E34,F34)</f>
         <v>Q20,,0.25</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="39"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="43" t="s">
+      <c r="B35" s="40"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="E35" s="27"/>
-      <c r="F35" s="28" t="n">
+      <c r="E35" s="28"/>
+      <c r="F35" s="29" t="n">
         <v>0.25</v>
       </c>
-      <c r="G35" s="29" t="s">
+      <c r="G35" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="H35" s="2" t="str">
+      <c r="H35" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G35,E35,F35)</f>
         <v>Q21,,0.25</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="39"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="25" t="s">
+      <c r="B36" s="40"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="E36" s="30"/>
-      <c r="F36" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="2" t="s">
+      <c r="E36" s="31"/>
+      <c r="F36" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H36" s="2" t="str">
+      <c r="H36" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G36,E36,F36)</f>
         <v>Q22,,1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="39"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="26" t="s">
+      <c r="B37" s="40"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="E37" s="27"/>
-      <c r="F37" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="29" t="s">
+      <c r="E37" s="28"/>
+      <c r="F37" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="H37" s="2" t="str">
+      <c r="H37" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G37,E37,F37)</f>
         <v>Q23,,1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="39"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="25" t="s">
+      <c r="B38" s="40"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="E38" s="30"/>
-      <c r="F38" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="E38" s="31"/>
+      <c r="F38" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H38" s="2" t="str">
+      <c r="H38" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G38,E38,F38)</f>
         <v>Q24,,1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="39"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="26" t="s">
+      <c r="B39" s="40"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="E39" s="27"/>
-      <c r="F39" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="29" t="s">
+      <c r="E39" s="28"/>
+      <c r="F39" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="H39" s="2" t="str">
+      <c r="H39" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G39,E39,F39)</f>
         <v>Q25,,1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="39"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="25" t="s">
+      <c r="B40" s="40"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="E40" s="30"/>
-      <c r="F40" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="E40" s="31"/>
+      <c r="F40" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H40" s="2" t="str">
+      <c r="H40" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G40,E40,F40)</f>
-        <v>Q26,,0.5</v>
+        <v>Q26,,1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="39"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="45" t="s">
+      <c r="B41" s="40"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="E41" s="27"/>
-      <c r="F41" s="46" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G41" s="29" t="s">
+      <c r="E41" s="28"/>
+      <c r="F41" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="H41" s="2" t="str">
+      <c r="H41" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G41,E41,F41)</f>
-        <v>Q27,,0.5</v>
+        <v>Q27,,1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="47" t="s">
+      <c r="B42" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C42" s="48" t="s">
+      <c r="C42" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="D42" s="48" t="s">
+      <c r="D42" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="E42" s="30"/>
-      <c r="F42" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="E42" s="31"/>
+      <c r="F42" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H42" s="2" t="str">
+      <c r="H42" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G42,E42,F42)</f>
         <v>Q28,,1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="47"/>
-      <c r="C43" s="48"/>
-      <c r="D43" s="26" t="s">
+      <c r="B43" s="48"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="E43" s="27"/>
-      <c r="F43" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="29" t="s">
+      <c r="E43" s="28"/>
+      <c r="F43" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="H43" s="2" t="str">
+      <c r="H43" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G43,E43,F43)</f>
         <v>Q29,,1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="47"/>
-      <c r="C44" s="48"/>
-      <c r="D44" s="25" t="s">
+      <c r="B44" s="48"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="E44" s="30"/>
-      <c r="F44" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="2" t="s">
+      <c r="E44" s="31"/>
+      <c r="F44" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H44" s="2" t="str">
+      <c r="H44" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G44,E44,F44)</f>
         <v>Q30,,1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="47"/>
-      <c r="C45" s="25" t="s">
+      <c r="B45" s="48"/>
+      <c r="C45" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="D45" s="26" t="s">
+      <c r="D45" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="E45" s="27"/>
-      <c r="F45" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="29" t="s">
+      <c r="E45" s="28"/>
+      <c r="F45" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="H45" s="2" t="str">
+      <c r="H45" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G45,E45,F45)</f>
         <v>Q31,,1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="47"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25" t="s">
+      <c r="B46" s="48"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="E46" s="30"/>
-      <c r="F46" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G46" s="2" t="s">
+      <c r="E46" s="31"/>
+      <c r="F46" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H46" s="2" t="str">
+      <c r="H46" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G46,E46,F46)</f>
-        <v>Q32,,0.5</v>
+        <v>Q32,,1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="47"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="26" t="s">
+      <c r="B47" s="48"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="E47" s="27"/>
-      <c r="F47" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G47" s="29" t="s">
+      <c r="E47" s="28"/>
+      <c r="F47" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="H47" s="2" t="str">
+      <c r="H47" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G47,E47,F47)</f>
-        <v>Q33,,0.5</v>
+        <v>Q33,,1</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="47"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="25" t="s">
+      <c r="B48" s="48"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="E48" s="30"/>
-      <c r="F48" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="2" t="s">
+      <c r="E48" s="31"/>
+      <c r="F48" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H48" s="2" t="str">
+      <c r="H48" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G48,E48,F48)</f>
         <v>Q34,,1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="47"/>
-      <c r="C49" s="37" t="s">
+      <c r="B49" s="48"/>
+      <c r="C49" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="D49" s="26" t="s">
+      <c r="D49" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="E49" s="27"/>
-      <c r="F49" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="29" t="s">
+      <c r="E49" s="28"/>
+      <c r="F49" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="H49" s="2" t="str">
+      <c r="H49" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G49,E49,F49)</f>
         <v>Q35,,1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="47"/>
-      <c r="C50" s="37"/>
-      <c r="D50" s="25" t="s">
+      <c r="B50" s="48"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="E50" s="30"/>
-      <c r="F50" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" s="2" t="s">
+      <c r="E50" s="31"/>
+      <c r="F50" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H50" s="2" t="str">
+      <c r="H50" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G50,E50,F50)</f>
         <v>Q36,,1</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="47"/>
-      <c r="C51" s="37"/>
-      <c r="D51" s="50" t="s">
+      <c r="B51" s="48"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="51" t="s">
         <v>99</v>
       </c>
-      <c r="E51" s="27"/>
-      <c r="F51" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="29" t="s">
+      <c r="E51" s="28"/>
+      <c r="F51" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="H51" s="2" t="str">
+      <c r="H51" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G51,E51,F51)</f>
         <v>Q37,,1</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="52" t="s">
+      <c r="B52" s="53" t="s">
         <v>101</v>
       </c>
-      <c r="C52" s="40" t="s">
+      <c r="C52" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="40" t="s">
+      <c r="D52" s="41" t="s">
         <v>103</v>
       </c>
-      <c r="E52" s="30"/>
-      <c r="F52" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="2" t="s">
+      <c r="E52" s="31"/>
+      <c r="F52" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="H52" s="2" t="str">
+      <c r="H52" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G52,E52,F52)</f>
         <v>Q38,,1</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="52"/>
-      <c r="C53" s="40"/>
-      <c r="D53" s="26" t="s">
+      <c r="B53" s="53"/>
+      <c r="C53" s="41"/>
+      <c r="D53" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E53" s="27"/>
-      <c r="F53" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="29" t="s">
+      <c r="E53" s="28"/>
+      <c r="F53" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="H53" s="2" t="str">
+      <c r="H53" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G53,E53,F53)</f>
         <v>Q39,,1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B54" s="52"/>
-      <c r="C54" s="40"/>
-      <c r="D54" s="25" t="s">
+      <c r="B54" s="53"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="E54" s="30"/>
-      <c r="F54" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G54" s="2" t="s">
+      <c r="E54" s="31"/>
+      <c r="F54" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="H54" s="2" t="str">
+      <c r="H54" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G54,E54,F54)</f>
-        <v>Q40,,0.5</v>
+        <v>Q40,,1</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="52"/>
-      <c r="C55" s="40"/>
-      <c r="D55" s="26" t="s">
+      <c r="B55" s="53"/>
+      <c r="C55" s="41"/>
+      <c r="D55" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="E55" s="27"/>
-      <c r="F55" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G55" s="29" t="s">
+      <c r="E55" s="28"/>
+      <c r="F55" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="H55" s="2" t="str">
+      <c r="H55" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G55,E55,F55)</f>
-        <v>Q41,,0.5</v>
+        <v>Q41,,1</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="52"/>
-      <c r="C56" s="32" t="s">
+      <c r="B56" s="53"/>
+      <c r="C56" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="D56" s="25" t="s">
+      <c r="D56" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="E56" s="30"/>
-      <c r="F56" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G56" s="2" t="s">
+      <c r="E56" s="31"/>
+      <c r="F56" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H56" s="2" t="str">
+      <c r="H56" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G56,E56,F56)</f>
         <v>Q42,,1</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="52"/>
-      <c r="C57" s="32"/>
-      <c r="D57" s="26" t="s">
+      <c r="B57" s="53"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="E57" s="27"/>
-      <c r="F57" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" s="29" t="s">
+      <c r="E57" s="28"/>
+      <c r="F57" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="H57" s="2" t="str">
+      <c r="H57" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G57,E57,F57)</f>
         <v>Q43,,1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="52"/>
-      <c r="C58" s="32"/>
-      <c r="D58" s="32" t="s">
+      <c r="B58" s="53"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="E58" s="30"/>
-      <c r="F58" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G58" s="2" t="s">
+      <c r="E58" s="31"/>
+      <c r="F58" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="H58" s="2" t="str">
+      <c r="H58" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G58,E58,F58)</f>
         <v>Q44,,1</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B59" s="47" t="s">
+      <c r="B59" s="48" t="s">
         <v>118</v>
       </c>
-      <c r="C59" s="47" t="s">
+      <c r="C59" s="48" t="s">
         <v>118</v>
       </c>
-      <c r="D59" s="35" t="s">
+      <c r="D59" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="E59" s="27"/>
-      <c r="F59" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" s="29" t="s">
+      <c r="E59" s="28"/>
+      <c r="F59" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="H59" s="2" t="str">
+      <c r="H59" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G59,E59,F59)</f>
         <v>Q45,,1</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B60" s="47"/>
-      <c r="C60" s="47"/>
-      <c r="D60" s="25" t="s">
+      <c r="B60" s="48"/>
+      <c r="C60" s="48"/>
+      <c r="D60" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="E60" s="30"/>
-      <c r="F60" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" s="2" t="s">
+      <c r="E60" s="31"/>
+      <c r="F60" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H60" s="2" t="str">
+      <c r="H60" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G60,E60,F60)</f>
         <v>Q46,,1</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B61" s="47"/>
-      <c r="C61" s="47"/>
-      <c r="D61" s="50" t="s">
+      <c r="B61" s="48"/>
+      <c r="C61" s="48"/>
+      <c r="D61" s="51" t="s">
         <v>123</v>
       </c>
-      <c r="E61" s="27"/>
-      <c r="F61" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="29" t="s">
+      <c r="E61" s="28"/>
+      <c r="F61" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="H61" s="2" t="str">
+      <c r="H61" s="3" t="str">
         <f aca="false">_xlfn.TEXTJOIN(",",FALSE(),G61,E61,F61)</f>
         <v>Q47,,1</v>
       </c>

</xml_diff>